<commit_message>
7/9 book keeper update
</commit_message>
<xml_diff>
--- a/SSRM Sample Book Keeper.xlsx
+++ b/SSRM Sample Book Keeper.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/marcusjl18/2026/Summer 2026/SSRM Files/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/marcusjl18/Research/SSRM 2026/Github/2026_SSRM_Duluth_Complex/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FCEACE29-CFC6-1A43-8236-2C6491A394B0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B3E70F4F-A60D-2C48-85F8-06AE02C609E1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="1080" yWindow="1160" windowWidth="27640" windowHeight="16220" xr2:uid="{F08D8A90-EBA7-134B-81EE-EBCE2C82C132}"/>
   </bookViews>
@@ -1153,10 +1153,13 @@
         <v>0</v>
       </c>
       <c r="J3" s="6" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K3" s="6" t="b">
-        <v>0</v>
+        <v>1</v>
+      </c>
+      <c r="N3" s="6" t="b">
+        <v>1</v>
       </c>
       <c r="O3" t="s">
         <v>184</v>
@@ -1235,15 +1238,18 @@
         <v>1</v>
       </c>
       <c r="J5" s="6" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K5" s="6" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L5" s="6" t="b">
         <v>1</v>
       </c>
       <c r="M5" s="6" t="b">
+        <v>1</v>
+      </c>
+      <c r="N5" s="6" t="b">
         <v>1</v>
       </c>
     </row>
@@ -1270,10 +1276,10 @@
         <v>170</v>
       </c>
       <c r="H6" s="6" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I6" s="6" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J6" s="6" t="b">
         <v>1</v>
@@ -3436,10 +3442,13 @@
         <v>0</v>
       </c>
       <c r="J63" s="6" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K63" s="6" t="b">
-        <v>0</v>
+        <v>1</v>
+      </c>
+      <c r="N63" s="6" t="b">
+        <v>1</v>
       </c>
       <c r="O63" t="s">
         <v>183</v>

</xml_diff>

<commit_message>
7/14 Book Keeper update
</commit_message>
<xml_diff>
--- a/SSRM Sample Book Keeper.xlsx
+++ b/SSRM Sample Book Keeper.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/marcusjl18/Research/SSRM 2026/Github/2026_SSRM_Duluth_Complex/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B3E70F4F-A60D-2C48-85F8-06AE02C609E1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5E86D62C-9502-F048-9078-7CAA443134F6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1080" yWindow="1160" windowWidth="27640" windowHeight="16220" xr2:uid="{F08D8A90-EBA7-134B-81EE-EBCE2C82C132}"/>
+    <workbookView xWindow="1620" yWindow="1160" windowWidth="27640" windowHeight="16220" xr2:uid="{F08D8A90-EBA7-134B-81EE-EBCE2C82C132}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="524" uniqueCount="185">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="531" uniqueCount="193">
   <si>
     <t>sample name</t>
   </si>
@@ -594,16 +594,47 @@
   </si>
   <si>
     <t>core too short for pmag saw</t>
+  </si>
+  <si>
+    <t>b mostly sulfide, c not, d completely sulfide</t>
+  </si>
+  <si>
+    <t>d contains plag chip</t>
+  </si>
+  <si>
+    <t>d contains oxide-rich plag chip</t>
+  </si>
+  <si>
+    <t>d contains hematite chip</t>
+  </si>
+  <si>
+    <t>d contains olivine chip</t>
+  </si>
+  <si>
+    <t>d contains albite chip</t>
+  </si>
+  <si>
+    <t>d contains hornblende chip</t>
+  </si>
+  <si>
+    <t>vsm sample d?</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color rgb="FF000000"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -659,7 +690,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
@@ -673,6 +704,7 @@
         </ext>
       </extLst>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1024,7 +1056,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BF8020B1-EECE-A849-93C3-8BFACC09541E}">
-  <dimension ref="A1:O85"/>
+  <dimension ref="A1:P85"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="5" max="5" width="16.6640625" customWidth="1"/>
@@ -1032,11 +1064,11 @@
     <col min="8" max="8" width="14.6640625" customWidth="1"/>
     <col min="10" max="10" width="16" customWidth="1"/>
     <col min="12" max="13" width="11.83203125" customWidth="1"/>
-    <col min="14" max="14" width="14.1640625" customWidth="1"/>
-    <col min="15" max="15" width="22.5" customWidth="1"/>
+    <col min="14" max="15" width="14.1640625" customWidth="1"/>
+    <col min="16" max="16" width="22.5" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -1080,10 +1112,13 @@
         <v>179</v>
       </c>
       <c r="O1" t="s">
+        <v>192</v>
+      </c>
+      <c r="P1" t="s">
         <v>180</v>
       </c>
     </row>
-    <row r="2" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>6</v>
       </c>
@@ -1124,7 +1159,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>11</v>
       </c>
@@ -1161,11 +1196,11 @@
       <c r="N3" s="6" t="b">
         <v>1</v>
       </c>
-      <c r="O3" t="s">
+      <c r="P3" t="s">
         <v>184</v>
       </c>
     </row>
-    <row r="4" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>13</v>
       </c>
@@ -1209,7 +1244,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="5" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
         <v>15</v>
       </c>
@@ -1252,8 +1287,14 @@
       <c r="N5" s="6" t="b">
         <v>1</v>
       </c>
-    </row>
-    <row r="6" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="O5" s="6" t="b">
+        <v>1</v>
+      </c>
+      <c r="P5" s="7" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="6" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
         <v>16</v>
       </c>
@@ -1287,11 +1328,8 @@
       <c r="K6" s="6" t="b">
         <v>1</v>
       </c>
-      <c r="O6" t="s">
-        <v>184</v>
-      </c>
-    </row>
-    <row r="7" spans="1:15" x14ac:dyDescent="0.2">
+    </row>
+    <row r="7" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
         <v>18</v>
       </c>
@@ -1329,7 +1367,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="8" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
         <v>21</v>
       </c>
@@ -1370,7 +1408,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="9" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
         <v>25</v>
       </c>
@@ -1405,7 +1443,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="10" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
         <v>28</v>
       </c>
@@ -1440,7 +1478,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="11" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
         <v>30</v>
       </c>
@@ -1475,7 +1513,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="12" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
         <v>31</v>
       </c>
@@ -1512,11 +1550,14 @@
       <c r="N12" s="6" t="b">
         <v>1</v>
       </c>
-      <c r="O12" t="s">
+      <c r="O12" s="6" t="b">
+        <v>1</v>
+      </c>
+      <c r="P12" t="s">
         <v>181</v>
       </c>
     </row>
-    <row r="13" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
         <v>33</v>
       </c>
@@ -1557,7 +1598,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="14" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
         <v>34</v>
       </c>
@@ -1595,7 +1636,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="15" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
         <v>38</v>
       </c>
@@ -1630,7 +1671,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="16" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
         <v>40</v>
       </c>
@@ -1665,7 +1706,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="17" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
         <v>41</v>
       </c>
@@ -1703,7 +1744,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="18" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
         <v>44</v>
       </c>
@@ -1738,7 +1779,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="19" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
         <v>47</v>
       </c>
@@ -1773,7 +1814,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="20" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
         <v>48</v>
       </c>
@@ -1811,7 +1852,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="21" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A21" t="s">
         <v>50</v>
       </c>
@@ -1849,7 +1890,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="22" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A22" t="s">
         <v>51</v>
       </c>
@@ -1893,7 +1934,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="23" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A23" t="s">
         <v>52</v>
       </c>
@@ -1934,7 +1975,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="24" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A24" t="s">
         <v>54</v>
       </c>
@@ -1972,7 +2013,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="25" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A25" t="s">
         <v>58</v>
       </c>
@@ -2016,7 +2057,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="26" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A26" t="s">
         <v>60</v>
       </c>
@@ -2051,7 +2092,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="27" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A27" t="s">
         <v>62</v>
       </c>
@@ -2092,7 +2133,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="28" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A28" t="s">
         <v>64</v>
       </c>
@@ -2129,11 +2170,14 @@
       <c r="N28" s="6" t="b">
         <v>1</v>
       </c>
-      <c r="O28" t="s">
-        <v>181</v>
-      </c>
-    </row>
-    <row r="29" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="O28" s="6" t="b">
+        <v>1</v>
+      </c>
+      <c r="P28" t="s">
+        <v>185</v>
+      </c>
+    </row>
+    <row r="29" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A29" t="s">
         <v>66</v>
       </c>
@@ -2170,8 +2214,14 @@
       <c r="N29" s="6" t="b">
         <v>1</v>
       </c>
-    </row>
-    <row r="30" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="O29" s="6" t="b">
+        <v>1</v>
+      </c>
+      <c r="P29" t="s">
+        <v>187</v>
+      </c>
+    </row>
+    <row r="30" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A30" t="s">
         <v>69</v>
       </c>
@@ -2208,8 +2258,14 @@
       <c r="N30" s="6" t="b">
         <v>1</v>
       </c>
-    </row>
-    <row r="31" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="O30" s="6" t="b">
+        <v>1</v>
+      </c>
+      <c r="P30" t="s">
+        <v>186</v>
+      </c>
+    </row>
+    <row r="31" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A31" t="s">
         <v>72</v>
       </c>
@@ -2246,8 +2302,14 @@
       <c r="N31" s="6" t="b">
         <v>1</v>
       </c>
-    </row>
-    <row r="32" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="O31" s="6" t="b">
+        <v>1</v>
+      </c>
+      <c r="P31" s="7" t="s">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="32" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A32" t="s">
         <v>75</v>
       </c>
@@ -2288,7 +2350,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="33" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="33" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A33" t="s">
         <v>77</v>
       </c>
@@ -2332,7 +2394,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="34" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="34" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A34" t="s">
         <v>80</v>
       </c>
@@ -2367,7 +2429,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="35" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="35" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A35" t="s">
         <v>81</v>
       </c>
@@ -2411,7 +2473,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="36" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="36" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A36" t="s">
         <v>83</v>
       </c>
@@ -2449,7 +2511,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="37" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="37" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A37" t="s">
         <v>84</v>
       </c>
@@ -2486,8 +2548,14 @@
       <c r="N37" s="6" t="b">
         <v>1</v>
       </c>
-    </row>
-    <row r="38" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="O37" s="6" t="b">
+        <v>1</v>
+      </c>
+      <c r="P37" t="s">
+        <v>186</v>
+      </c>
+    </row>
+    <row r="38" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A38" t="s">
         <v>86</v>
       </c>
@@ -2525,7 +2593,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="39" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="39" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A39" t="s">
         <v>88</v>
       </c>
@@ -2560,7 +2628,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="40" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="40" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A40" t="s">
         <v>89</v>
       </c>
@@ -2595,7 +2663,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="41" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="41" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A41" t="s">
         <v>90</v>
       </c>
@@ -2633,7 +2701,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="42" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="42" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A42" t="s">
         <v>91</v>
       </c>
@@ -2668,7 +2736,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="43" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="43" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A43" t="s">
         <v>94</v>
       </c>
@@ -2703,7 +2771,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="44" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="44" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A44" t="s">
         <v>97</v>
       </c>
@@ -2738,7 +2806,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="45" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="45" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A45" t="s">
         <v>99</v>
       </c>
@@ -2782,7 +2850,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="46" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="46" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A46" t="s">
         <v>102</v>
       </c>
@@ -2820,7 +2888,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="47" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="47" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A47" t="s">
         <v>104</v>
       </c>
@@ -2858,7 +2926,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="48" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="48" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A48" t="s">
         <v>106</v>
       </c>
@@ -2899,7 +2967,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="49" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="49" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A49" t="s">
         <v>108</v>
       </c>
@@ -2934,7 +3002,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="50" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="50" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A50" t="s">
         <v>112</v>
       </c>
@@ -2971,8 +3039,14 @@
       <c r="N50" s="6" t="b">
         <v>1</v>
       </c>
-    </row>
-    <row r="51" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="O50" s="6" t="b">
+        <v>1</v>
+      </c>
+      <c r="P50" s="7" t="s">
+        <v>191</v>
+      </c>
+    </row>
+    <row r="51" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A51" t="s">
         <v>115</v>
       </c>
@@ -3016,7 +3090,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="52" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="52" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A52" t="s">
         <v>116</v>
       </c>
@@ -3054,7 +3128,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="53" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="53" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A53" t="s">
         <v>118</v>
       </c>
@@ -3089,7 +3163,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="54" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="54" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A54" t="s">
         <v>119</v>
       </c>
@@ -3124,7 +3198,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="55" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="55" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A55" t="s">
         <v>120</v>
       </c>
@@ -3159,7 +3233,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="56" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="56" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A56" t="s">
         <v>121</v>
       </c>
@@ -3197,7 +3271,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="57" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="57" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A57" t="s">
         <v>122</v>
       </c>
@@ -3232,7 +3306,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="58" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="58" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A58" t="s">
         <v>123</v>
       </c>
@@ -3267,7 +3341,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="59" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="59" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A59" t="s">
         <v>124</v>
       </c>
@@ -3302,7 +3376,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="60" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="60" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A60" t="s">
         <v>125</v>
       </c>
@@ -3337,7 +3411,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="61" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="61" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A61" t="s">
         <v>127</v>
       </c>
@@ -3375,7 +3449,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="62" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="62" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A62" t="s">
         <v>129</v>
       </c>
@@ -3413,7 +3487,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="63" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="63" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A63" t="s">
         <v>130</v>
       </c>
@@ -3450,11 +3524,11 @@
       <c r="N63" s="6" t="b">
         <v>1</v>
       </c>
-      <c r="O63" t="s">
+      <c r="P63" t="s">
         <v>183</v>
       </c>
     </row>
-    <row r="64" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="64" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A64" t="s">
         <v>133</v>
       </c>
@@ -3489,7 +3563,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="65" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="65" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A65" t="s">
         <v>134</v>
       </c>
@@ -3527,7 +3601,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="66" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="66" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A66" t="s">
         <v>136</v>
       </c>
@@ -3562,7 +3636,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="67" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="67" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A67" t="s">
         <v>137</v>
       </c>
@@ -3597,7 +3671,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="68" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="68" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A68" t="s">
         <v>139</v>
       </c>
@@ -3632,7 +3706,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="69" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="69" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A69" t="s">
         <v>140</v>
       </c>
@@ -3673,7 +3747,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="70" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="70" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A70" t="s">
         <v>141</v>
       </c>
@@ -3708,7 +3782,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="71" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="71" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A71" t="s">
         <v>142</v>
       </c>
@@ -3746,7 +3820,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="72" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="72" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A72" t="s">
         <v>145</v>
       </c>
@@ -3781,7 +3855,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="73" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="73" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A73" t="s">
         <v>147</v>
       </c>
@@ -3816,7 +3890,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="74" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="74" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A74" t="s">
         <v>150</v>
       </c>
@@ -3851,7 +3925,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="75" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="75" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A75" t="s">
         <v>151</v>
       </c>
@@ -3886,7 +3960,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="76" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="76" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A76" t="s">
         <v>152</v>
       </c>
@@ -3921,7 +3995,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="77" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="77" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A77" t="s">
         <v>153</v>
       </c>
@@ -3962,7 +4036,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="78" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="78" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A78" t="s">
         <v>154</v>
       </c>
@@ -3999,8 +4073,14 @@
       <c r="N78" s="6" t="b">
         <v>1</v>
       </c>
-    </row>
-    <row r="79" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="O78" s="6" t="b">
+        <v>1</v>
+      </c>
+      <c r="P78" s="7" t="s">
+        <v>188</v>
+      </c>
+    </row>
+    <row r="79" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A79" t="s">
         <v>156</v>
       </c>
@@ -4035,7 +4115,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="80" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="80" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A80" t="s">
         <v>159</v>
       </c>

</xml_diff>

<commit_message>
7/15 Book Keeper Update
</commit_message>
<xml_diff>
--- a/SSRM Sample Book Keeper.xlsx
+++ b/SSRM Sample Book Keeper.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/marcusjl18/Research/SSRM 2026/Github/2026_SSRM_Duluth_Complex/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5E86D62C-9502-F048-9078-7CAA443134F6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F44C57B2-A298-9943-B7DC-82F71D1D4AA2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="1620" yWindow="1160" windowWidth="27640" windowHeight="16220" xr2:uid="{F08D8A90-EBA7-134B-81EE-EBCE2C82C132}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="531" uniqueCount="193">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="533" uniqueCount="194">
   <si>
     <t>sample name</t>
   </si>
@@ -590,9 +590,6 @@
     <t>TS polished</t>
   </si>
   <si>
-    <t>Unable to make pmag sample</t>
-  </si>
-  <si>
     <t>core too short for pmag saw</t>
   </si>
   <si>
@@ -618,6 +615,12 @@
   </si>
   <si>
     <t>vsm sample d?</t>
+  </si>
+  <si>
+    <t>Unable to make pmag sample, d contains serpentine chip</t>
+  </si>
+  <si>
+    <t>d contains serpentine chip</t>
   </si>
 </sst>
 </file>
@@ -1112,7 +1115,7 @@
         <v>179</v>
       </c>
       <c r="O1" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="P1" t="s">
         <v>180</v>
@@ -1197,7 +1200,7 @@
         <v>1</v>
       </c>
       <c r="P3" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
     </row>
     <row r="4" spans="1:16" x14ac:dyDescent="0.2">
@@ -1291,7 +1294,7 @@
         <v>1</v>
       </c>
       <c r="P5" s="7" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
     </row>
     <row r="6" spans="1:16" x14ac:dyDescent="0.2">
@@ -2174,7 +2177,7 @@
         <v>1</v>
       </c>
       <c r="P28" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
     </row>
     <row r="29" spans="1:16" x14ac:dyDescent="0.2">
@@ -2218,7 +2221,7 @@
         <v>1</v>
       </c>
       <c r="P29" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
     </row>
     <row r="30" spans="1:16" x14ac:dyDescent="0.2">
@@ -2262,7 +2265,7 @@
         <v>1</v>
       </c>
       <c r="P30" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
     </row>
     <row r="31" spans="1:16" x14ac:dyDescent="0.2">
@@ -2306,7 +2309,7 @@
         <v>1</v>
       </c>
       <c r="P31" s="7" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
     </row>
     <row r="32" spans="1:16" x14ac:dyDescent="0.2">
@@ -2552,7 +2555,7 @@
         <v>1</v>
       </c>
       <c r="P37" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
     </row>
     <row r="38" spans="1:16" x14ac:dyDescent="0.2">
@@ -3043,7 +3046,7 @@
         <v>1</v>
       </c>
       <c r="P50" s="7" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
     </row>
     <row r="51" spans="1:16" x14ac:dyDescent="0.2">
@@ -3127,6 +3130,12 @@
       <c r="N52" s="6" t="b">
         <v>1</v>
       </c>
+      <c r="O52" s="6" t="b">
+        <v>1</v>
+      </c>
+      <c r="P52" t="s">
+        <v>193</v>
+      </c>
     </row>
     <row r="53" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A53" t="s">
@@ -3340,6 +3349,15 @@
       <c r="K58" s="6" t="b">
         <v>1</v>
       </c>
+      <c r="N58" s="6" t="b">
+        <v>1</v>
+      </c>
+      <c r="O58" s="6" t="b">
+        <v>1</v>
+      </c>
+      <c r="P58" t="s">
+        <v>193</v>
+      </c>
     </row>
     <row r="59" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A59" t="s">
@@ -3524,8 +3542,11 @@
       <c r="N63" s="6" t="b">
         <v>1</v>
       </c>
+      <c r="O63" s="6" t="b">
+        <v>1</v>
+      </c>
       <c r="P63" t="s">
-        <v>183</v>
+        <v>192</v>
       </c>
     </row>
     <row r="64" spans="1:16" x14ac:dyDescent="0.2">
@@ -4077,7 +4098,7 @@
         <v>1</v>
       </c>
       <c r="P78" s="7" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
     </row>
     <row r="79" spans="1:16" x14ac:dyDescent="0.2">

</xml_diff>

<commit_message>
7/15 Final Book Keeper Update
</commit_message>
<xml_diff>
--- a/SSRM Sample Book Keeper.xlsx
+++ b/SSRM Sample Book Keeper.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/marcusjl18/Research/SSRM 2026/Github/2026_SSRM_Duluth_Complex/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F44C57B2-A298-9943-B7DC-82F71D1D4AA2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{82063302-469D-1745-BA15-C84B7E0659A6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="1620" yWindow="1160" windowWidth="27640" windowHeight="16220" xr2:uid="{F08D8A90-EBA7-134B-81EE-EBCE2C82C132}"/>
   </bookViews>
@@ -4076,8 +4076,8 @@
       <c r="F78" t="s">
         <v>27</v>
       </c>
-      <c r="G78" s="2" t="s">
-        <v>174</v>
+      <c r="G78" s="1" t="s">
+        <v>170</v>
       </c>
       <c r="H78" s="6" t="b">
         <v>1</v>

</xml_diff>